<commit_message>
Add FCFF/WACC valuation and enterprise-to-equity bridge
</commit_message>
<xml_diff>
--- a/tsla-proforma-model/output/TSLA_model.xlsx
+++ b/tsla-proforma-model/output/TSLA_model.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Historical Financials" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Forecast" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Valuation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Scenarios" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Checks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Financials" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-06T22:05</t>
+          <t>Generated: 2026-10-19T10:54</t>
         </is>
       </c>
     </row>
@@ -536,34 +536,41 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>FCFF implied value per share: $27.22</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>DISCLAIMER: Educational and research use only. This model is not investment advice and is not a recommendation to buy, sell or hold TSLA or any other security. Forecasts are hypothetical, depend on judgment-based assumptions that are clearly labelled, and may be materially wrong. Historical data are taken from Tesla's SEC filings; verify all figures against the original documents before relying on them. Past performance does not predict future results.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Data status this session:</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  [info] seed: Seed data compiled 2026-09-24 loaded (used wherever live data is unavailable).</t>
+          <t>Data status this session:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [info] seed: Seed data compiled 2026-09-24 loaded (used wherever live data is unavailable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  [fallback] network: Offline mode selected; seed data only.</t>
         </is>
@@ -37437,7 +37444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:N128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -37447,10 +37454,13 @@
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="39" customWidth="1" min="10" max="10"/>
     <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -38440,115 +38450,1078 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>SECONDARY cross-check: trading multiples (not the primary valuation)</t>
+          <t>Discounted FCFF (WACC)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Method</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Multiple</t>
+          <t>EBIT</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Implied value per share</t>
+          <t>Tax on EBIT</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>D&amp;A</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>SBC added back</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Capex</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Increase in NWC</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>FCFF</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Less H1-2026 actual (already in cash)</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>FCFF valued</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Discount period (yrs)</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>Discount factor</t>
+        </is>
+      </c>
+      <c r="N65" s="3" t="inlineStr">
+        <is>
+          <t>PV</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Peer median EV / revenue (LFY) x FY2026E revenue</t>
-        </is>
-      </c>
-      <c r="B66" s="19" t="n">
-        <v>1.999295763873452</v>
-      </c>
-      <c r="C66" s="17" t="n">
-        <v>68.06784294533719</v>
+          <t>FY2026E (H2 only)</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="n">
+        <v>2152.191000000003</v>
+      </c>
+      <c r="C66" s="4" t="n">
+        <v>-559.5696600000007</v>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>1592.621340000002</v>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>6520.67</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>4343.871</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="H66" s="4" t="n">
+        <v>1428.268297780818</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>-11114.56936221918</v>
+      </c>
+      <c r="J66" s="5" t="n">
+        <v>70.26336061627353</v>
+      </c>
+      <c r="K66" s="4" t="n">
+        <v>-11044.3060016029</v>
+      </c>
+      <c r="L66" s="14" t="n">
+        <v>0.2683093771389459</v>
+      </c>
+      <c r="M66" s="16" t="n">
+        <v>0.9739764751171032</v>
+      </c>
+      <c r="N66" s="4" t="n">
+        <v>-10756.89422955586</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Peer median P/E (profitable peers) x FY2026E net income</t>
-        </is>
-      </c>
-      <c r="B67" s="19" t="n">
-        <v>25.62435544230885</v>
-      </c>
-      <c r="C67" s="17" t="n">
-        <v>18.48208468412002</v>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="n">
+        <v>1124.434699999998</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>-281.1086749999995</v>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>843.3260249999985</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>8941.1829</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>4554.664000000001</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>-22000</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>1737.0914518022</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>-5923.735623197801</v>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="4" t="n">
+        <v>-5923.735623197801</v>
+      </c>
+      <c r="L67" s="14" t="n">
+        <v>1.267624914442163</v>
+      </c>
+      <c r="M67" s="16" t="n">
+        <v>0.8828712012370196</v>
+      </c>
+      <c r="N67" s="4" t="n">
+        <v>-5229.895585463168</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Forward P/E 15x (judgment) x FY2027E EPS</t>
-        </is>
-      </c>
-      <c r="B68" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="C68" s="17" t="n">
-        <v>6.220258906991879</v>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>1822.818276999998</v>
+      </c>
+      <c r="C68" s="4" t="n">
+        <v>-437.4763864799996</v>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>1385.341890519999</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>10649.229123</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>4820.541224</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="H68" s="4" t="n">
+        <v>2141.524454173381</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>996.6366916933803</v>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="4" t="n">
+        <v>996.6366916933803</v>
+      </c>
+      <c r="L68" s="14" t="n">
+        <v>2.269678302532512</v>
+      </c>
+      <c r="M68" s="16" t="n">
+        <v>0.8000725707350484</v>
+      </c>
+      <c r="N68" s="4" t="n">
+        <v>797.3816800119967</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Forward P/E 40x (judgment) x FY2027E EPS</t>
-        </is>
-      </c>
-      <c r="B69" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="C69" s="17" t="n">
-        <v>16.58735708531168</v>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>3743.348978509992</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>-860.9702650572982</v>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2882.378713452694</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>11615.22933701</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>5060.83405248</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="H69" s="4" t="n">
+        <v>2251.910996615174</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>5810.353099557869</v>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="4" t="n">
+        <v>5810.353099557869</v>
+      </c>
+      <c r="L69" s="14" t="n">
+        <v>3.268993839835729</v>
+      </c>
+      <c r="M69" s="16" t="n">
+        <v>0.7252341813663572</v>
+      </c>
+      <c r="N69" s="4" t="n">
+        <v>4213.866673607327</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="n">
+        <v>5843.368106426882</v>
+      </c>
+      <c r="C70" s="4" t="n">
+        <v>-1343.974664478183</v>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>4499.3934419487</v>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>12195.6495231987</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>5218.1358898368</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="H70" s="4" t="n">
+        <v>2115.64458473619</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>9028.823439720385</v>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="4" t="n">
+        <v>9028.823439720385</v>
+      </c>
+      <c r="L70" s="14" t="n">
+        <v>4.268309377138946</v>
+      </c>
+      <c r="M70" s="16" t="n">
+        <v>0.6573961376265059</v>
+      </c>
+      <c r="N70" s="4" t="n">
+        <v>5935.513656583845</v>
+      </c>
+    </row>
+    <row r="71"/>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>2031 terminal FCFF bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>FY2031</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>EBIT (FY2030E x (1+g))</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="n">
+        <v>5843.368106426882</v>
+      </c>
+      <c r="C74" s="4" t="n">
+        <v>6018.669149619689</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>- Tax on EBIT</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="n">
+        <v>-1343.974664478183</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>-1384.293904412528</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <f> NOPAT</f>
+        <v/>
+      </c>
+      <c r="B76" s="4" t="n">
+        <v>4499.3934419487</v>
+      </c>
+      <c r="C76" s="4" t="n">
+        <v>4634.37524520716</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>+ D&amp;A (grown at g)</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>12195.6495231987</v>
+      </c>
+      <c r="C77" s="4" t="n">
+        <v>12561.51900889466</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>+ SBC (if added back)</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="n">
+        <v>5218.1358898368</v>
+      </c>
+      <c r="C78" s="4" t="n">
+        <v>5374.679966531904</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>- Capex (terminal capex/D&amp;A x D&amp;A)</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="C79" s="4" t="n">
+        <v>-14445.74686022886</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>- Increase in NWC (NWC x g)</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>2115.64458473619</v>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>759.4031935532329</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <f> FCFF</f>
+        <v/>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>9028.823439720385</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>8884.230553958099</v>
+      </c>
+    </row>
+    <row r="82"/>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>FCFF enterprise-value-to-equity bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>PV of FCFF (H2 2026 - 2030)</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="n">
+        <v>-5040.027804815864</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="n">
+        <v>79715.55088509197</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Enterprise value</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="n">
+        <v>74675.52308027611</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Cash &amp; ST investments (30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="n">
+        <v>43524</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Less: minimum operating cash</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="n">
+        <v>-15513.825</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Excess cash</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="n">
+        <v>28010.175</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Digital assets (30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="n">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SpaceX equity investment (carrying value)</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="n">
+        <v>3007</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Total non-operating assets</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="n">
+        <v>31691.175</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Debt (ex-finance leases, 30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="n">
+        <v>-9061</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Finance lease liabilities (30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="n">
+        <v>-281</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Revolver (30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="n">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Noncontrolling interests incl. redeemable NCI (30-Jun-2026)</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="n">
+        <v>-661</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Equity value</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="n">
+        <v>96363.69808027611</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Diluted shares (M)</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="n">
+        <v>3540</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Implied value per share ($)</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n">
+        <v>27.22138363849608</v>
+      </c>
+    </row>
+    <row r="101"/>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>FCFF-to-FCFE reconciliation (residual is not forced to zero)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>The recurring -$60M residual is net income attributable to noncontrolling interests, which FCFE to common excludes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>FCFF</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>- After-tax interest expense</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>+ After-tax interest income</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>+ Net borrowing</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>Implied FCFE</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>Model FCFE</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>Residual</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="n">
+        <v>-11114.56936221918</v>
+      </c>
+      <c r="C105" s="4" t="n">
+        <v>-254.12784</v>
+      </c>
+      <c r="D105" s="4" t="n">
+        <v>1274.803106</v>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>920</v>
+      </c>
+      <c r="F105" s="4" t="n">
+        <v>-9173.894096219179</v>
+      </c>
+      <c r="G105" s="4" t="n">
+        <v>-9233.894096219181</v>
+      </c>
+      <c r="H105" s="5" t="n">
+        <v>-60.00000000000182</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="n">
+        <v>-5923.735623197801</v>
+      </c>
+      <c r="C106" s="4" t="n">
+        <v>-290.157</v>
+      </c>
+      <c r="D106" s="4" t="n">
+        <v>988.0503306283725</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>-80</v>
+      </c>
+      <c r="F106" s="4" t="n">
+        <v>-5305.842292569429</v>
+      </c>
+      <c r="G106" s="4" t="n">
+        <v>-5365.842292569429</v>
+      </c>
+      <c r="H106" s="4" t="n">
+        <v>-60</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="n">
+        <v>996.6366916933803</v>
+      </c>
+      <c r="C107" s="4" t="n">
+        <v>-294.02576</v>
+      </c>
+      <c r="D107" s="4" t="n">
+        <v>867.6258854707576</v>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>420</v>
+      </c>
+      <c r="F107" s="4" t="n">
+        <v>1990.236817164138</v>
+      </c>
+      <c r="G107" s="4" t="n">
+        <v>1930.236817164139</v>
+      </c>
+      <c r="H107" s="5" t="n">
+        <v>-59.99999999999864</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="n">
+        <v>5810.353099557869</v>
+      </c>
+      <c r="C108" s="4" t="n">
+        <v>-313.67952</v>
+      </c>
+      <c r="D108" s="4" t="n">
+        <v>963.348745397102</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>-2580</v>
+      </c>
+      <c r="F108" s="4" t="n">
+        <v>3880.022324954972</v>
+      </c>
+      <c r="G108" s="4" t="n">
+        <v>3820.022324954971</v>
+      </c>
+      <c r="H108" s="5" t="n">
+        <v>-60.00000000000091</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="n">
+        <v>9028.823439720385</v>
+      </c>
+      <c r="C109" s="4" t="n">
+        <v>-234.75452</v>
+      </c>
+      <c r="D109" s="4" t="n">
+        <v>1104.551247534522</v>
+      </c>
+      <c r="E109" s="4" t="n">
+        <v>420</v>
+      </c>
+      <c r="F109" s="4" t="n">
+        <v>10318.62016725491</v>
+      </c>
+      <c r="G109" s="4" t="n">
+        <v>10258.62016725491</v>
+      </c>
+      <c r="H109" s="4" t="n">
+        <v>-60</v>
+      </c>
+    </row>
+    <row r="110"/>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
+        <is>
+          <t>FCFF WACC x terminal growth ($/share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>WACC \ terminal growth</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="B113" s="17" t="n">
+        <v>28.78633606759022</v>
+      </c>
+      <c r="C113" s="17" t="n">
+        <v>33.89259403688229</v>
+      </c>
+      <c r="D113" s="17" t="n">
+        <v>41.04135519389113</v>
+      </c>
+      <c r="E113" s="17" t="n">
+        <v>51.76449692940442</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>9%</t>
+        </is>
+      </c>
+      <c r="B114" s="17" t="n">
+        <v>24.90612892456651</v>
+      </c>
+      <c r="C114" s="17" t="n">
+        <v>28.70402546050117</v>
+      </c>
+      <c r="D114" s="17" t="n">
+        <v>33.76788750841403</v>
+      </c>
+      <c r="E114" s="17" t="n">
+        <v>40.85729437549205</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="B115" s="17" t="n">
+        <v>21.90684407510707</v>
+      </c>
+      <c r="C115" s="17" t="n">
+        <v>24.83455982957329</v>
+      </c>
+      <c r="D115" s="17" t="n">
+        <v>28.59876579960125</v>
+      </c>
+      <c r="E115" s="17" t="n">
+        <v>33.61770709297188</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>11%</t>
+        </is>
+      </c>
+      <c r="B116" s="17" t="n">
+        <v>19.52361159964041</v>
+      </c>
+      <c r="C116" s="17" t="n">
+        <v>21.84378851173586</v>
+      </c>
+      <c r="D116" s="17" t="n">
+        <v>24.74400965185515</v>
+      </c>
+      <c r="E116" s="17" t="n">
+        <v>28.47286540343711</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="B117" s="17" t="n">
+        <v>17.58790187193779</v>
+      </c>
+      <c r="C117" s="17" t="n">
+        <v>19.46749550819456</v>
+      </c>
+      <c r="D117" s="17" t="n">
+        <v>21.76477661917504</v>
+      </c>
+      <c r="E117" s="17" t="n">
+        <v>24.63637800790065</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="B118" s="17" t="n">
+        <v>15.98738262098042</v>
+      </c>
+      <c r="C118" s="17" t="n">
+        <v>17.53756845184733</v>
+      </c>
+      <c r="D118" s="17" t="n">
+        <v>19.39779144888761</v>
+      </c>
+      <c r="E118" s="17" t="n">
+        <v>21.67139733415908</v>
+      </c>
+    </row>
+    <row r="119"/>
+    <row r="120">
+      <c r="A120" s="1" t="inlineStr">
+        <is>
+          <t>SECONDARY cross-check: trading multiples (not the primary valuation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Implied value per share</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Peer median EV / revenue (LFY) x FY2026E revenue</t>
+        </is>
+      </c>
+      <c r="B122" s="19" t="n">
+        <v>1.999295763873452</v>
+      </c>
+      <c r="C122" s="17" t="n">
+        <v>68.06784294533719</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Peer median P/E (profitable peers) x FY2026E net income</t>
+        </is>
+      </c>
+      <c r="B123" s="19" t="n">
+        <v>25.62435544230885</v>
+      </c>
+      <c r="C123" s="17" t="n">
+        <v>18.48208468412002</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Forward P/E 15x (judgment) x FY2027E EPS</t>
+        </is>
+      </c>
+      <c r="B124" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C124" s="17" t="n">
+        <v>6.220258906991879</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Forward P/E 40x (judgment) x FY2027E EPS</t>
+        </is>
+      </c>
+      <c r="B125" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="C125" s="17" t="n">
+        <v>16.58735708531168</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
           <t>Market-implied P/E on FY2026E net income (price x shares / NI)</t>
         </is>
       </c>
-      <c r="B70" s="19" t="n">
+      <c r="B126" s="19" t="n">
         <v>524.4220341864972</v>
       </c>
-      <c r="C70" s="17" t="n">
+      <c r="C126" s="17" t="n">
         <v>378.25</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="127">
+      <c r="A127" t="inlineStr">
         <is>
           <t>Market-implied P/E on FY2027E net income</t>
         </is>
       </c>
-      <c r="B71" s="19" t="n">
+      <c r="B127" s="19" t="n">
         <v>903.9883221293445</v>
       </c>
-      <c r="C71" s="17" t="n">
+      <c r="C127" s="17" t="n">
         <v>378.25</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="128">
+      <c r="A128" t="inlineStr">
         <is>
           <t>Market-implied EV / FY2026E revenue</t>
         </is>
       </c>
-      <c r="B72" s="19" t="n">
+      <c r="B128" s="19" t="n">
         <v>12.61606663733799</v>
       </c>
-      <c r="C72" s="17" t="n">
+      <c r="C128" s="17" t="n">
         <v>378.25</v>
       </c>
     </row>

</xml_diff>